<commit_message>
feat: add WhatsApp integration, file attachments, Cc/Bcc email fields, and autocomplete dropdowns
</commit_message>
<xml_diff>
--- a/csm_company_mappings (14).xlsx
+++ b/csm_company_mappings (14).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1286"/>
+  <dimension ref="A1:O1288"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -60843,9 +60843,103 @@
         <v/>
       </c>
     </row>
+    <row r="1287">
+      <c r="A1287" t="str">
+        <v>1836</v>
+      </c>
+      <c r="B1287" t="str">
+        <v>uvx</v>
+      </c>
+      <c r="C1287" t="str">
+        <v/>
+      </c>
+      <c r="D1287" t="str">
+        <v/>
+      </c>
+      <c r="E1287" t="str">
+        <v>deepa</v>
+      </c>
+      <c r="F1287" t="str">
+        <v/>
+      </c>
+      <c r="G1287" t="str">
+        <v/>
+      </c>
+      <c r="H1287" t="str">
+        <v/>
+      </c>
+      <c r="I1287" t="str">
+        <v/>
+      </c>
+      <c r="J1287" t="str">
+        <v/>
+      </c>
+      <c r="K1287" t="str">
+        <v/>
+      </c>
+      <c r="L1287" t="str">
+        <v/>
+      </c>
+      <c r="M1287" t="str">
+        <v/>
+      </c>
+      <c r="N1287" t="str">
+        <v/>
+      </c>
+      <c r="O1287" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="str">
+        <v>1837</v>
+      </c>
+      <c r="B1288" t="str">
+        <v>xyz</v>
+      </c>
+      <c r="C1288" t="str">
+        <v/>
+      </c>
+      <c r="D1288" t="str">
+        <v/>
+      </c>
+      <c r="E1288" t="str">
+        <v>deepanker gupta</v>
+      </c>
+      <c r="F1288" t="str">
+        <v>7665619297</v>
+      </c>
+      <c r="G1288" t="str">
+        <v>deepanker.gupta@flick2know.com</v>
+      </c>
+      <c r="H1288" t="str">
+        <v/>
+      </c>
+      <c r="I1288" t="str">
+        <v/>
+      </c>
+      <c r="J1288" t="str">
+        <v/>
+      </c>
+      <c r="K1288" t="str">
+        <v/>
+      </c>
+      <c r="L1288" t="str">
+        <v/>
+      </c>
+      <c r="M1288" t="str">
+        <v/>
+      </c>
+      <c r="N1288" t="str">
+        <v/>
+      </c>
+      <c r="O1288" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1286"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1288"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>